<commit_message>
Update preprocessing report outputs
</commit_message>
<xml_diff>
--- a/mepram/preprocessing_report/tables/clinician_variable_dictionary.xlsx
+++ b/mepram/preprocessing_report/tables/clinician_variable_dictionary.xlsx
@@ -236,7 +236,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -323,7 +323,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -410,7 +410,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Recoded in tbl_paciente from mujer_gestante, center, dag: fill missing values with False after joining center and previous-infection data. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Recoded in tbl_paciente from mujer_gestante, center, dag: fill missing values with False after joining center and previous-infection data. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Recoded in tbl_paciente from mujer_gestante, center, dag: fill missing values with False after joining center and previous-infection data. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Recoded in tbl_paciente from mujer_gestante, center, dag: fill missing values with False after joining center and previous-infection data. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Recoded in tbl_paciente from mujer_gestante, center, dag: fill missing values with False after joining center and previous-infection data. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Recoded in tbl_paciente from mujer_gestante, center, dag: fill missing values with False after joining center and previous-infection data. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -4238,7 +4238,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -6152,7 +6152,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -6413,7 +6413,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
@@ -7022,7 +7022,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
@@ -7370,7 +7370,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -7457,7 +7457,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
@@ -7544,7 +7544,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -7718,7 +7718,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -7805,7 +7805,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -7979,7 +7979,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P92" t="inlineStr">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P94" t="inlineStr">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P95" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P96" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P98" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
@@ -8849,7 +8849,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
@@ -9023,7 +9023,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -9110,7 +9110,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -9197,7 +9197,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
@@ -9284,7 +9284,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P108" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -9719,7 +9719,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
@@ -9806,7 +9806,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
@@ -10067,7 +10067,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -10241,7 +10241,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -10328,7 +10328,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -10415,7 +10415,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_comorbilidad from tipo_cancer, tipo_hepatopatia: one-hot encode categorical comorbidity variables. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P137" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>Transformed in tbl_sepsis from proteina_c_reactiva, sofa, respiracion, snc_glasgow, cardiovascular, ... (9 source variables): extract numeric values from mixed text fields, including '= N score' score strings. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Transformed in tbl_sepsis from proteina_c_reactiva, sofa, respiracion, snc_glasgow, cardiovascular, ... (9 source variables): extract numeric values from mixed text fields, including '= N score' score strings. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P148" t="inlineStr">
@@ -13112,7 +13112,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>Created in tbl_sepsis from proteina_c_reactiva: create ordinal quartile category after IQR outlier removal; IQR limits lower=-104.72, upper=154.84; outliers replaced=507; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 0.0 to 5.4; 1: 5.4 to 14.274000000000001; 2: 14.274000000000001 to 28.198; 3: 28.198 to 154.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_sepsis from proteina_c_reactiva: create ordinal quartile category after IQR outlier removal; IQR limits lower=-104.72, upper=154.84; outliers replaced=507; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 0.0 to 5.4; 1: 5.4 to 14.274000000000001; 2: 14.274000000000001 to 28.198; 3: 28.198 to 154.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P150" t="inlineStr">
@@ -13808,7 +13808,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>Recoded in tbl_signos from tension_arterial: binary hypotension flag recomputed after numeric cleaning: 1 if tension_arterial &lt;= 100.0, 0 otherwise, and preserve original value if tension_arterial is missing. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Recoded in tbl_signos from tension_arterial: binary hypotension flag recomputed after numeric cleaning: 1 if tension_arterial &lt;= 100.0, 0 otherwise, and preserve original value if tension_arterial is missing. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P158" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>Created in tbl_signos from temperatura: create ordinal quartile category after IQR outlier removal; IQR limits lower=31.799999999999997, upper=43.00000000000001; outliers replaced=0; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 32.0 to 36.6; 1: 36.6 to 37.4; 2: 37.4 to 38.2; 3: 38.2 to 41.2. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_signos from temperatura: create ordinal quartile category after IQR outlier removal; IQR limits lower=31.799999999999997, upper=43.00000000000001; outliers replaced=0; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 32.0 to 36.6; 1: 36.6 to 37.4; 2: 37.4 to 38.2; 3: 38.2 to 41.2. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
@@ -14156,7 +14156,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>Created in tbl_signos from frec_respiratoria: create ordinal quartile category after IQR outlier removal; IQR limits lower=-4.0, upper=45.0; outliers replaced=9; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 7.0 to 17.0; 1: 17.0 to 20.0; 2: 20.0 to 24.0; 3: 24.0 to 45.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_signos from frec_respiratoria: create ordinal quartile category after IQR outlier removal; IQR limits lower=-4.0, upper=45.0; outliers replaced=9; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 7.0 to 17.0; 1: 17.0 to 20.0; 2: 20.0 to 24.0; 3: 24.0 to 45.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P162" t="inlineStr">
@@ -14243,7 +14243,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>Created in tbl_signos from frec_cardiaca: create ordinal quartile category after IQR outlier removal; IQR limits lower=-3.0, upper=200.0; outliers replaced=0; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 33.0 to 84.0; 1: 84.0 to 98.0; 2: 98.0 to 113.0; 3: 113.0 to 200.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_signos from frec_cardiaca: create ordinal quartile category after IQR outlier removal; IQR limits lower=-3.0, upper=200.0; outliers replaced=0; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 33.0 to 84.0; 1: 84.0 to 98.0; 2: 98.0 to 113.0; 3: 113.0 to 200.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -14330,7 +14330,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>Created in tbl_signos from tension_arterial: create ordinal quartile category after IQR outlier removal; IQR limits lower=-13.0, upper=242.5; outliers replaced=0; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 49.0 to 96.5; 1: 96.5 to 114.0; 2: 114.0 to 133.0; 3: 133.0 to 226.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_signos from tension_arterial: create ordinal quartile category after IQR outlier removal; IQR limits lower=-13.0, upper=242.5; outliers replaced=0; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 49.0 to 96.5; 1: 96.5 to 114.0; 2: 114.0 to 133.0; 3: 133.0 to 226.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -14417,7 +14417,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>Created in tbl_signos from saturacion_o2: create ordinal quartile category after IQR outlier removal; IQR limits lower=81.0, upper=109.0; outliers replaced=70; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 81.0 to 93.0; 1: 93.0 to 96.0; 2: 96.0 to 97.0; 3: 97.0 to 100.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_signos from saturacion_o2: create ordinal quartile category after IQR outlier removal; IQR limits lower=81.0, upper=109.0; outliers replaced=70; pd.qcut(q=4, labels 0-3, duplicates='drop'); categories: 0: 81.0 to 93.0; 1: 93.0 to 96.0; 2: 96.0 to 97.0; 3: 97.0 to 100.0. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P165" t="inlineStr">
@@ -16766,7 +16766,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P192" t="inlineStr">
@@ -16853,7 +16853,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P193" t="inlineStr">
@@ -16940,7 +16940,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P194" t="inlineStr">
@@ -17027,7 +17027,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
@@ -17114,7 +17114,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P196" t="inlineStr">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P197" t="inlineStr">
@@ -17288,7 +17288,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P198" t="inlineStr">
@@ -17375,7 +17375,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P199" t="inlineStr">
@@ -17462,7 +17462,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P200" t="inlineStr">
@@ -17549,7 +17549,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, bmr_infec_previa: create organism-specific previous-infection BMR binary flags using max bmr_infec_previa per patient/admission/organism. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P201" t="inlineStr">
@@ -17636,7 +17636,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P202" t="inlineStr">
@@ -17723,7 +17723,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P203" t="inlineStr">
@@ -17810,7 +17810,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P204" t="inlineStr">
@@ -17897,7 +17897,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P205" t="inlineStr">
@@ -17984,7 +17984,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P206" t="inlineStr">
@@ -18071,7 +18071,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P207" t="inlineStr">
@@ -18158,7 +18158,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P208" t="inlineStr">
@@ -18245,7 +18245,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P209" t="inlineStr">
@@ -18332,7 +18332,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P210" t="inlineStr">
@@ -18419,7 +18419,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_infecciones_previas from grupo_microorganismo, feno_resist_infec_prev: create organism-specific previous-infection phenotype tuples using non-zero deduplicated feno_resist_infec_prev codes. Transformed in tbl_infecciones_previas from missing patient/admission rows after previous-infection aggregation: complete output to all master patient/admissions; fill absent previous-infection exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P211" t="inlineStr">
@@ -23900,7 +23900,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
@@ -23987,7 +23987,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P275" t="inlineStr">
@@ -24074,7 +24074,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P276" t="inlineStr">
@@ -24161,7 +24161,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P277" t="inlineStr">
@@ -24248,7 +24248,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
@@ -24335,7 +24335,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P279" t="inlineStr">
@@ -24422,7 +24422,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P280" t="inlineStr">
@@ -24509,7 +24509,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
@@ -24596,7 +24596,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
@@ -24683,7 +24683,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, bmr_colonizador: create organism-specific colonization BMR binary flags using max bmr_colonizador per patient/admission/organism. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -24770,7 +24770,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -24944,7 +24944,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P286" t="inlineStr">
@@ -25031,7 +25031,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
@@ -25118,7 +25118,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
@@ -25205,7 +25205,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -25292,7 +25292,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -25379,7 +25379,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -25466,7 +25466,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
@@ -25553,7 +25553,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_colonizaciones_previas from microorganism_colonizador_grupo, feno_resist_colo: create organism-specific colonization phenotype tuples using non-zero deduplicated feno_resist_colo codes. Transformed in tbl_colonizaciones_previas from missing patient/admission rows after colonization aggregation: complete output to all master patient/admissions; fill absent colonization exposure/count columns with 0 and organism-specific phenotype tuples with NEGATIVE. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
@@ -25901,7 +25901,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
@@ -25988,7 +25988,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
@@ -26075,7 +26075,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
@@ -26162,7 +26162,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P300" t="inlineStr">
@@ -26249,7 +26249,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P301" t="inlineStr">
@@ -26336,7 +26336,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P302" t="inlineStr">
@@ -26423,7 +26423,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P303" t="inlineStr">
@@ -26510,7 +26510,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P304" t="inlineStr">
@@ -26597,7 +26597,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P305" t="inlineStr">
@@ -26684,7 +26684,7 @@
       </c>
       <c r="O306" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo: pivot grouped hemoculture organisms to binary columns per patient/admission. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P306" t="inlineStr">
@@ -26771,7 +26771,7 @@
       </c>
       <c r="O307" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P307" t="inlineStr">
@@ -26858,7 +26858,7 @@
       </c>
       <c r="O308" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P308" t="inlineStr">
@@ -26945,7 +26945,7 @@
       </c>
       <c r="O309" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P309" t="inlineStr">
@@ -27032,7 +27032,7 @@
       </c>
       <c r="O310" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P310" t="inlineStr">
@@ -27119,7 +27119,7 @@
       </c>
       <c r="O311" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P311" t="inlineStr">
@@ -27206,7 +27206,7 @@
       </c>
       <c r="O312" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P312" t="inlineStr">
@@ -27293,7 +27293,7 @@
       </c>
       <c r="O313" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P313" t="inlineStr">
@@ -27380,7 +27380,7 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P314" t="inlineStr">
@@ -27467,7 +27467,7 @@
       </c>
       <c r="O315" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P315" t="inlineStr">
@@ -27554,7 +27554,7 @@
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, bmr_etiologia: create organism-specific hemoculture BMR binary flags using max bmr_etiologia per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P316" t="inlineStr">
@@ -27641,7 +27641,7 @@
       </c>
       <c r="O317" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P317" t="inlineStr">
@@ -27728,7 +27728,7 @@
       </c>
       <c r="O318" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P318" t="inlineStr">
@@ -27815,7 +27815,7 @@
       </c>
       <c r="O319" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P319" t="inlineStr">
@@ -27902,7 +27902,7 @@
       </c>
       <c r="O320" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P320" t="inlineStr">
@@ -27989,7 +27989,7 @@
       </c>
       <c r="O321" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P321" t="inlineStr">
@@ -28076,7 +28076,7 @@
       </c>
       <c r="O322" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P322" t="inlineStr">
@@ -28163,7 +28163,7 @@
       </c>
       <c r="O323" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P323" t="inlineStr">
@@ -28250,7 +28250,7 @@
       </c>
       <c r="O324" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P324" t="inlineStr">
@@ -28337,7 +28337,7 @@
       </c>
       <c r="O325" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P325" t="inlineStr">
@@ -28424,7 +28424,7 @@
       </c>
       <c r="O326" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo, fenotipo_resistencia: create organism-specific hemoculture phenotype tuples using non-zero deduplicated fenotipo_resistencia codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P326" t="inlineStr">
@@ -28511,7 +28511,7 @@
       </c>
       <c r="O327" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P327" t="inlineStr">
@@ -28598,7 +28598,7 @@
       </c>
       <c r="O328" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P328" t="inlineStr">
@@ -28685,7 +28685,7 @@
       </c>
       <c r="O329" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P329" t="inlineStr">
@@ -28772,7 +28772,7 @@
       </c>
       <c r="O330" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P330" t="inlineStr">
@@ -28859,7 +28859,7 @@
       </c>
       <c r="O331" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P331" t="inlineStr">
@@ -28946,7 +28946,7 @@
       </c>
       <c r="O332" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P332" t="inlineStr">
@@ -29033,7 +29033,7 @@
       </c>
       <c r="O333" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P333" t="inlineStr">
@@ -29120,7 +29120,7 @@
       </c>
       <c r="O334" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P334" t="inlineStr">
@@ -29207,7 +29207,7 @@
       </c>
       <c r="O335" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P335" t="inlineStr">
@@ -29294,7 +29294,7 @@
       </c>
       <c r="O336" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P336" t="inlineStr">
@@ -29381,7 +29381,7 @@
       </c>
       <c r="O337" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo: pivot grouped other emergency culture organisms to count columns per patient/admission. Transformed in tbl_otros_cultivos_en_urgencias from tipo_cultivo, otro_cult_microorganismo: drop duplicate patient/admission/culture-type/organism rows before pivoting organism counts. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P337" t="inlineStr">
@@ -29468,7 +29468,7 @@
       </c>
       <c r="O338" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P338" t="inlineStr">
@@ -29555,7 +29555,7 @@
       </c>
       <c r="O339" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P339" t="inlineStr">
@@ -29642,7 +29642,7 @@
       </c>
       <c r="O340" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P340" t="inlineStr">
@@ -29729,7 +29729,7 @@
       </c>
       <c r="O341" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P341" t="inlineStr">
@@ -29816,7 +29816,7 @@
       </c>
       <c r="O342" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P342" t="inlineStr">
@@ -29903,7 +29903,7 @@
       </c>
       <c r="O343" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P343" t="inlineStr">
@@ -29990,7 +29990,7 @@
       </c>
       <c r="O344" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P344" t="inlineStr">
@@ -30077,7 +30077,7 @@
       </c>
       <c r="O345" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P345" t="inlineStr">
@@ -30164,7 +30164,7 @@
       </c>
       <c r="O346" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P346" t="inlineStr">
@@ -30251,7 +30251,7 @@
       </c>
       <c r="O347" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P347" t="inlineStr">
@@ -30338,7 +30338,7 @@
       </c>
       <c r="O348" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, bmr_etiologia_otros: create organism-specific other-culture BMR binary flags using max bmr_etiologia_otros per patient/admission/organism. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P348" t="inlineStr">
@@ -30425,7 +30425,7 @@
       </c>
       <c r="O349" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P349" t="inlineStr">
@@ -30512,7 +30512,7 @@
       </c>
       <c r="O350" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P350" t="inlineStr">
@@ -30599,7 +30599,7 @@
       </c>
       <c r="O351" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P351" t="inlineStr">
@@ -30686,7 +30686,7 @@
       </c>
       <c r="O352" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P352" t="inlineStr">
@@ -30773,7 +30773,7 @@
       </c>
       <c r="O353" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P353" t="inlineStr">
@@ -30860,7 +30860,7 @@
       </c>
       <c r="O354" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P354" t="inlineStr">
@@ -30947,7 +30947,7 @@
       </c>
       <c r="O355" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P355" t="inlineStr">
@@ -31034,7 +31034,7 @@
       </c>
       <c r="O356" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P356" t="inlineStr">
@@ -31121,7 +31121,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P357" t="inlineStr">
@@ -31208,7 +31208,7 @@
       </c>
       <c r="O358" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P358" t="inlineStr">
@@ -31295,7 +31295,7 @@
       </c>
       <c r="O359" t="inlineStr">
         <is>
-          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in tbl_otros_cultivos_en_urgencias from otro_cult_microorganismo, fenotipo_resistencia_otros: create organism-specific other-culture phenotype tuples using non-zero deduplicated fenotipo_resistencia_otros codes. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P359" t="inlineStr">
@@ -31382,7 +31382,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P360" t="inlineStr">
@@ -31469,7 +31469,7 @@
       </c>
       <c r="O361" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P361" t="inlineStr">
@@ -31556,7 +31556,7 @@
       </c>
       <c r="O362" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P362" t="inlineStr">
@@ -31643,7 +31643,7 @@
       </c>
       <c r="O363" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P363" t="inlineStr">
@@ -31730,7 +31730,7 @@
       </c>
       <c r="O364" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P364" t="inlineStr">
@@ -31817,7 +31817,7 @@
       </c>
       <c r="O365" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P365" t="inlineStr">
@@ -31904,7 +31904,7 @@
       </c>
       <c r="O366" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P366" t="inlineStr">
@@ -31991,7 +31991,7 @@
       </c>
       <c r="O367" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P367" t="inlineStr">
@@ -32078,7 +32078,7 @@
       </c>
       <c r="O368" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P368" t="inlineStr">
@@ -32165,7 +32165,7 @@
       </c>
       <c r="O369" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P369" t="inlineStr">
@@ -32252,7 +32252,7 @@
       </c>
       <c r="O370" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_*_binary, otros_cult_*: sum hemoculture organism binaries and other-emergency-culture organism counts into combined urgent-culture count columns. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P370" t="inlineStr">
@@ -32339,7 +32339,7 @@
       </c>
       <c r="O371" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P371" t="inlineStr">
@@ -32426,7 +32426,7 @@
       </c>
       <c r="O372" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P372" t="inlineStr">
@@ -32513,7 +32513,7 @@
       </c>
       <c r="O373" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P373" t="inlineStr">
@@ -32600,7 +32600,7 @@
       </c>
       <c r="O374" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P374" t="inlineStr">
@@ -32687,7 +32687,7 @@
       </c>
       <c r="O375" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P375" t="inlineStr">
@@ -32774,7 +32774,7 @@
       </c>
       <c r="O376" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P376" t="inlineStr">
@@ -32861,7 +32861,7 @@
       </c>
       <c r="O377" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P377" t="inlineStr">
@@ -32948,7 +32948,7 @@
       </c>
       <c r="O378" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P378" t="inlineStr">
@@ -33035,7 +33035,7 @@
       </c>
       <c r="O379" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P379" t="inlineStr">
@@ -33122,7 +33122,7 @@
       </c>
       <c r="O380" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P380" t="inlineStr">
@@ -33209,7 +33209,7 @@
       </c>
       <c r="O381" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P381" t="inlineStr">
@@ -33296,7 +33296,7 @@
       </c>
       <c r="O382" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P382" t="inlineStr">
@@ -33383,7 +33383,7 @@
       </c>
       <c r="O383" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P383" t="inlineStr">
@@ -33470,7 +33470,7 @@
       </c>
       <c r="O384" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P384" t="inlineStr">
@@ -33557,7 +33557,7 @@
       </c>
       <c r="O385" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P385" t="inlineStr">
@@ -33644,7 +33644,7 @@
       </c>
       <c r="O386" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P386" t="inlineStr">
@@ -33731,7 +33731,7 @@
       </c>
       <c r="O387" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P387" t="inlineStr">
@@ -33818,7 +33818,7 @@
       </c>
       <c r="O388" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P388" t="inlineStr">
@@ -33905,7 +33905,7 @@
       </c>
       <c r="O389" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P389" t="inlineStr">
@@ -33992,7 +33992,7 @@
       </c>
       <c r="O390" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in mepram/config/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="P390" t="inlineStr">

</xml_diff>